<commit_message>
Fill missing MRPs in 15-patient file from rate card; add consolidated all-patients final bill
- 17 missing-rate rows priced (NS 100ml, syringes, Tramadol, Xone, Pan,
  Sensoricaine Heavy, Adrenaline, blades, Plain Sheet, suction); subtotals,
  grand totals, margins and summary recomputed; changes highlighted yellow
- 17 rows remain unpriced (Cap+Mask, O2/equipment charges, TURP set, etc.)
- New BKAditya_AllPatients_FinalBill.xlsx: 29 patients (15 early + 13 June
  + Raju Mondal mediclaim) in one sheet, consolidated total ₹190,061.18

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YWgR3jd3MUcEXpU4s4WC54
</commit_message>
<xml_diff>
--- a/BKAditya_PatientBilling_FINAL.xlsx
+++ b/BKAditya_PatientBilling_FINAL.xlsx
@@ -382,7 +382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -570,6 +570,21 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -975,7 +990,7 @@
         </is>
       </c>
       <c r="E5" s="58" t="n">
-        <v>2275.46</v>
+        <v>2321.1</v>
       </c>
       <c r="F5" s="23" t="n">
         <v>1000</v>
@@ -984,19 +999,19 @@
         <v>1500</v>
       </c>
       <c r="H5" s="58" t="n">
-        <v>4775.46</v>
-      </c>
-      <c r="I5" s="22" t="n">
-        <v>971.1799999999999</v>
+        <v>4821.1</v>
+      </c>
+      <c r="I5" s="58" t="n">
+        <v>992.74</v>
       </c>
       <c r="J5" s="58" t="n">
-        <v>3804.28</v>
+        <v>3828.36</v>
       </c>
       <c r="K5" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="24" t="n">
-        <v>5</v>
+      <c r="L5" s="66" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -1150,8 +1165,8 @@
           <t>OT</t>
         </is>
       </c>
-      <c r="E9" s="31" t="n">
-        <v>2388.86</v>
+      <c r="E9" s="58" t="n">
+        <v>2420.33</v>
       </c>
       <c r="F9" s="32" t="n">
         <v>1000</v>
@@ -1159,20 +1174,20 @@
       <c r="G9" s="32" t="n">
         <v>1500</v>
       </c>
-      <c r="H9" s="31" t="n">
-        <v>4888.86</v>
-      </c>
-      <c r="I9" s="31" t="n">
-        <v>785.95</v>
-      </c>
-      <c r="J9" s="31" t="n">
-        <v>4102.91</v>
+      <c r="H9" s="58" t="n">
+        <v>4920.33</v>
+      </c>
+      <c r="I9" s="58" t="n">
+        <v>810.71</v>
+      </c>
+      <c r="J9" s="58" t="n">
+        <v>4109.62</v>
       </c>
       <c r="K9" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="24" t="n">
-        <v>1</v>
+      <c r="L9" s="66" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -1370,8 +1385,8 @@
           <t>Ward</t>
         </is>
       </c>
-      <c r="E14" s="27" t="n">
-        <v>418.25</v>
+      <c r="E14" s="58" t="n">
+        <v>439.25</v>
       </c>
       <c r="F14" s="28" t="n">
         <v>1000</v>
@@ -1379,20 +1394,20 @@
       <c r="G14" s="28" t="n">
         <v>1500</v>
       </c>
-      <c r="H14" s="27" t="n">
-        <v>2918.25</v>
-      </c>
-      <c r="I14" s="27" t="n">
-        <v>238.12</v>
-      </c>
-      <c r="J14" s="27" t="n">
-        <v>2680.13</v>
+      <c r="H14" s="58" t="n">
+        <v>2939.25</v>
+      </c>
+      <c r="I14" s="58" t="n">
+        <v>251.12</v>
+      </c>
+      <c r="J14" s="58" t="n">
+        <v>2688.13</v>
       </c>
       <c r="K14" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="24" t="n">
-        <v>2</v>
+      <c r="L14" s="66" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -1415,7 +1430,7 @@
         </is>
       </c>
       <c r="E15" s="58" t="n">
-        <v>5144.65</v>
+        <v>6217.77</v>
       </c>
       <c r="F15" s="32" t="n">
         <v>1000</v>
@@ -1424,19 +1439,19 @@
         <v>1500</v>
       </c>
       <c r="H15" s="58" t="n">
-        <v>7644.65</v>
-      </c>
-      <c r="I15" s="31" t="n">
-        <v>2363.35</v>
+        <v>8717.77</v>
+      </c>
+      <c r="I15" s="58" t="n">
+        <v>2548.62</v>
       </c>
       <c r="J15" s="58" t="n">
-        <v>5281.3</v>
-      </c>
-      <c r="K15" s="33" t="n">
-        <v>4</v>
-      </c>
-      <c r="L15" s="24" t="n">
-        <v>6</v>
+        <v>6169.15</v>
+      </c>
+      <c r="K15" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" s="66" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1458,8 +1473,8 @@
           <t>OT</t>
         </is>
       </c>
-      <c r="E16" s="31" t="n">
-        <v>1674.91</v>
+      <c r="E16" s="58" t="n">
+        <v>1741.55</v>
       </c>
       <c r="F16" s="32" t="n">
         <v>1000</v>
@@ -1467,20 +1482,20 @@
       <c r="G16" s="32" t="n">
         <v>1500</v>
       </c>
-      <c r="H16" s="31" t="n">
-        <v>4174.91</v>
-      </c>
-      <c r="I16" s="31" t="n">
-        <v>693.48</v>
-      </c>
-      <c r="J16" s="31" t="n">
-        <v>3481.43</v>
+      <c r="H16" s="58" t="n">
+        <v>4241.55</v>
+      </c>
+      <c r="I16" s="58" t="n">
+        <v>719.1900000000001</v>
+      </c>
+      <c r="J16" s="58" t="n">
+        <v>3522.36</v>
       </c>
       <c r="K16" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="L16" s="24" t="n">
-        <v>1</v>
+      <c r="L16" s="66" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1547,7 +1562,7 @@
         </is>
       </c>
       <c r="E18" s="58" t="n">
-        <v>1447.58</v>
+        <v>1526.78</v>
       </c>
       <c r="F18" s="32" t="n">
         <v>1000</v>
@@ -1556,19 +1571,19 @@
         <v>1500</v>
       </c>
       <c r="H18" s="58" t="n">
-        <v>3947.58</v>
-      </c>
-      <c r="I18" s="31" t="n">
-        <v>975.1799999999999</v>
+        <v>4026.78</v>
+      </c>
+      <c r="I18" s="58" t="n">
+        <v>1005.65</v>
       </c>
       <c r="J18" s="58" t="n">
-        <v>2972.4</v>
+        <v>3021.13</v>
       </c>
       <c r="K18" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="L18" s="24" t="n">
-        <v>2</v>
+      <c r="L18" s="66" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1591,7 +1606,7 @@
         </is>
       </c>
       <c r="E19" s="58" t="n">
-        <v>8107.76</v>
+        <v>10510.76</v>
       </c>
       <c r="F19" s="32" t="n">
         <v>1000</v>
@@ -1600,19 +1615,19 @@
         <v>1500</v>
       </c>
       <c r="H19" s="58" t="n">
-        <v>10607.76</v>
-      </c>
-      <c r="I19" s="31" t="n">
-        <v>4595.19</v>
+        <v>13010.76</v>
+      </c>
+      <c r="I19" s="58" t="n">
+        <v>4775.19</v>
       </c>
       <c r="J19" s="58" t="n">
-        <v>6012.57</v>
+        <v>8235.57</v>
       </c>
       <c r="K19" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="L19" s="24" t="n">
-        <v>8</v>
+      <c r="L19" s="66" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="20" ht="21.75" customHeight="1">
@@ -1625,7 +1640,7 @@
       <c r="C20" s="59" t="n"/>
       <c r="D20" s="59" t="n"/>
       <c r="E20" s="60" t="n">
-        <v>31449.22</v>
+        <v>35169.29</v>
       </c>
       <c r="F20" s="34" t="n">
         <v>15000</v>
@@ -1634,13 +1649,13 @@
         <v>22500</v>
       </c>
       <c r="H20" s="60" t="n">
-        <v>68949.22</v>
-      </c>
-      <c r="I20" s="34" t="n">
-        <v>15382</v>
+        <v>72669.28999999999</v>
+      </c>
+      <c r="I20" s="60" t="n">
+        <v>15862.77</v>
       </c>
       <c r="J20" s="60" t="n">
-        <v>53567.22</v>
+        <v>56806.52</v>
       </c>
       <c r="K20" s="35" t="n"/>
       <c r="L20" s="35" t="n"/>
@@ -2444,50 +2459,42 @@
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1">
-      <c r="A8" s="24" t="n">
+      <c r="A8" s="66" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>IV+ NS 100 Ml</t>
         </is>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="68" t="inlineStr">
         <is>
           <t>Normal Saline 100ml</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J8" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D8" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E8" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="G8" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="H8" s="69" t="n">
+        <v>13</v>
+      </c>
+      <c r="I8" s="69" t="n">
+        <v>13</v>
+      </c>
+      <c r="J8" s="68" t="inlineStr">
+        <is>
+          <t>SL3 / Vivek F-748</t>
         </is>
       </c>
     </row>
@@ -2502,12 +2509,12 @@
       <c r="D9" s="62" t="n"/>
       <c r="E9" s="62" t="n"/>
       <c r="F9" s="62" t="n"/>
-      <c r="G9" s="42" t="n">
-        <v>418.25</v>
+      <c r="G9" s="63" t="n">
+        <v>439.25</v>
       </c>
       <c r="H9" s="43" t="n"/>
-      <c r="I9" s="42" t="n">
-        <v>238.12</v>
+      <c r="I9" s="63" t="n">
+        <v>251.12</v>
       </c>
       <c r="J9" s="43" t="n"/>
     </row>
@@ -2627,12 +2634,12 @@
       <c r="D17" s="59" t="n"/>
       <c r="E17" s="59" t="n"/>
       <c r="F17" s="59" t="n"/>
-      <c r="G17" s="52" t="n">
-        <v>2918.25</v>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Total Cost: ₹238.12  |  Margin: ₹2,680.13</t>
+      <c r="G17" s="64" t="n">
+        <v>2939.25</v>
+      </c>
+      <c r="H17" s="65" t="inlineStr">
+        <is>
+          <t>Total Cost: ₹251.12  |  Margin: ₹2,688.13</t>
         </is>
       </c>
       <c r="I17" s="59" t="n"/>
@@ -2647,9 +2654,9 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 2 item(s) without MRP: Cap + Mask | IV+ NS 100 Ml</t>
+      <c r="A20" s="70" t="inlineStr">
+        <is>
+          <t>⚠ 1 item(s) without MRP: Cap + Mask</t>
         </is>
       </c>
     </row>
@@ -2868,46 +2875,42 @@
       </c>
     </row>
     <row r="7" ht="13.5" customHeight="1">
-      <c r="A7" s="24" t="n">
+      <c r="A7" s="66" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="40" t="inlineStr">
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>Inj. Adrenaline</t>
         </is>
       </c>
-      <c r="C7" s="40" t="n"/>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E7" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="41" t="inlineStr">
+      <c r="C7" s="68" t="n"/>
+      <c r="D7" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="69" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G7" s="69" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="H7" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="G7" s="41" t="inlineStr">
+      <c r="I7" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="H7" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I7" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J7" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="J7" s="68" t="inlineStr">
+        <is>
+          <t>SL43 / Stock file</t>
         </is>
       </c>
     </row>
@@ -3428,50 +3431,46 @@
       </c>
     </row>
     <row r="21" ht="13.5" customHeight="1">
-      <c r="A21" s="24" t="n">
+      <c r="A21" s="66" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="40" t="inlineStr">
+      <c r="B21" s="68" t="inlineStr">
         <is>
           <t>Surgical Blade 24 No.</t>
         </is>
       </c>
-      <c r="C21" s="40" t="inlineStr">
+      <c r="C21" s="68" t="inlineStr">
         <is>
           <t>Surgical blade</t>
         </is>
       </c>
-      <c r="D21" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E21" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="41" t="inlineStr">
+      <c r="D21" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E21" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="69" t="n">
+        <v>710</v>
+      </c>
+      <c r="G21" s="69" t="n">
+        <v>710</v>
+      </c>
+      <c r="H21" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="G21" s="41" t="inlineStr">
+      <c r="I21" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="H21" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I21" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J21" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="J21" s="68" t="inlineStr">
+        <is>
+          <t>⚠ Est. proxy — Blade No.20 rate SL82</t>
         </is>
       </c>
     </row>
@@ -3556,98 +3555,82 @@
       </c>
     </row>
     <row r="24" ht="13.5" customHeight="1">
-      <c r="A24" s="24" t="n">
+      <c r="A24" s="66" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="40" t="inlineStr">
+      <c r="B24" s="68" t="inlineStr">
         <is>
           <t>Inj. Xone</t>
         </is>
       </c>
-      <c r="C24" s="40" t="inlineStr">
+      <c r="C24" s="68" t="inlineStr">
         <is>
           <t>Ceftriaxone 1g</t>
         </is>
       </c>
-      <c r="D24" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E24" s="24" t="n">
+      <c r="D24" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E24" s="66" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G24" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H24" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I24" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J24" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="F24" s="69" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="G24" s="69" t="n">
+        <v>199.92</v>
+      </c>
+      <c r="H24" s="69" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="I24" s="69" t="n">
+        <v>77.13</v>
+      </c>
+      <c r="J24" s="68" t="inlineStr">
+        <is>
+          <t>SL16 / SSB S000068</t>
         </is>
       </c>
     </row>
     <row r="25" ht="13.5" customHeight="1">
-      <c r="A25" s="24" t="n">
+      <c r="A25" s="66" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="40" t="inlineStr">
+      <c r="B25" s="68" t="inlineStr">
         <is>
           <t>Inj. Pan</t>
         </is>
       </c>
-      <c r="C25" s="40" t="inlineStr">
+      <c r="C25" s="68" t="inlineStr">
         <is>
           <t>Pantoprazole</t>
         </is>
       </c>
-      <c r="D25" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E25" s="24" t="n">
+      <c r="D25" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E25" s="66" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G25" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H25" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I25" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J25" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="F25" s="69" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="G25" s="69" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="H25" s="69" t="n">
+        <v>41.07</v>
+      </c>
+      <c r="I25" s="69" t="n">
+        <v>82.14</v>
+      </c>
+      <c r="J25" s="68" t="inlineStr">
+        <is>
+          <t>SL33 / SSB S000135</t>
         </is>
       </c>
     </row>
@@ -3924,50 +3907,42 @@
       </c>
     </row>
     <row r="33" ht="13.5" customHeight="1">
-      <c r="A33" s="24" t="n">
+      <c r="A33" s="66" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="40" t="inlineStr">
+      <c r="B33" s="68" t="inlineStr">
         <is>
           <t>100ml NS</t>
         </is>
       </c>
-      <c r="C33" s="40" t="inlineStr">
+      <c r="C33" s="68" t="inlineStr">
         <is>
           <t>Normal Saline 100ml</t>
         </is>
       </c>
-      <c r="D33" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E33" s="24" t="n">
+      <c r="D33" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E33" s="66" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G33" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H33" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I33" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J33" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="F33" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="G33" s="69" t="n">
+        <v>42</v>
+      </c>
+      <c r="H33" s="69" t="n">
+        <v>13</v>
+      </c>
+      <c r="I33" s="69" t="n">
+        <v>26</v>
+      </c>
+      <c r="J33" s="68" t="inlineStr">
+        <is>
+          <t>SL3 / Vivek F-748</t>
         </is>
       </c>
     </row>
@@ -4471,11 +4446,11 @@
       <c r="E46" s="62" t="n"/>
       <c r="F46" s="62" t="n"/>
       <c r="G46" s="63" t="n">
-        <v>5144.65</v>
+        <v>6217.77</v>
       </c>
       <c r="H46" s="43" t="n"/>
-      <c r="I46" s="42" t="n">
-        <v>2363.35</v>
+      <c r="I46" s="63" t="n">
+        <v>2548.62</v>
       </c>
       <c r="J46" s="43" t="n"/>
     </row>
@@ -4596,11 +4571,11 @@
       <c r="E54" s="59" t="n"/>
       <c r="F54" s="59" t="n"/>
       <c r="G54" s="64" t="n">
-        <v>7644.65</v>
+        <v>8717.77</v>
       </c>
       <c r="H54" s="65" t="inlineStr">
         <is>
-          <t>Total Cost: ₹2,363.35  |  Margin: ₹5,281.30</t>
+          <t>Total Cost: ₹2,548.62  |  Margin: ₹6,169.15</t>
         </is>
       </c>
       <c r="I54" s="59" t="n"/>
@@ -4615,9 +4590,9 @@
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 6 item(s) without MRP: Inj. Pan | Cap + Mask | Inj. Xone | 100ml NS | Surgical Blade 24 No. | Inj. Adrenaline</t>
+      <c r="A57" s="70" t="inlineStr">
+        <is>
+          <t>⚠ 1 item(s) without MRP: Cap + Mask</t>
         </is>
       </c>
     </row>
@@ -4908,50 +4883,42 @@
       </c>
     </row>
     <row r="9" ht="13.5" customHeight="1">
-      <c r="A9" s="24" t="n">
+      <c r="A9" s="66" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="40" t="inlineStr">
+      <c r="B9" s="68" t="inlineStr">
         <is>
           <t>Inj. Xone (1g)</t>
         </is>
       </c>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="C9" s="68" t="inlineStr">
         <is>
           <t>Ceftriaxone</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G9" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H9" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I9" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J9" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D9" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E9" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="69" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="G9" s="69" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="H9" s="69" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="I9" s="69" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="J9" s="68" t="inlineStr">
+        <is>
+          <t>SL16 / SSB S000068</t>
         </is>
       </c>
     </row>
@@ -5630,12 +5597,12 @@
       <c r="D27" s="62" t="n"/>
       <c r="E27" s="62" t="n"/>
       <c r="F27" s="62" t="n"/>
-      <c r="G27" s="42" t="n">
-        <v>1674.91</v>
+      <c r="G27" s="63" t="n">
+        <v>1741.55</v>
       </c>
       <c r="H27" s="43" t="n"/>
-      <c r="I27" s="42" t="n">
-        <v>693.48</v>
+      <c r="I27" s="63" t="n">
+        <v>719.1900000000001</v>
       </c>
       <c r="J27" s="43" t="n"/>
     </row>
@@ -5755,12 +5722,12 @@
       <c r="D35" s="59" t="n"/>
       <c r="E35" s="59" t="n"/>
       <c r="F35" s="59" t="n"/>
-      <c r="G35" s="52" t="n">
-        <v>4174.91</v>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Total Cost: ₹693.48  |  Margin: ₹3,481.43</t>
+      <c r="G35" s="64" t="n">
+        <v>4241.55</v>
+      </c>
+      <c r="H35" s="65" t="inlineStr">
+        <is>
+          <t>Total Cost: ₹719.19  |  Margin: ₹3,522.36</t>
         </is>
       </c>
       <c r="I35" s="59" t="n"/>
@@ -5775,9 +5742,9 @@
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 1 item(s) without MRP: Inj. Xone (1g)</t>
+      <c r="A38" s="70" t="inlineStr">
+        <is>
+          <t>✓ All items now priced from Master Rate Card — no missing MRPs</t>
         </is>
       </c>
     </row>
@@ -5785,8 +5752,8 @@
   <mergeCells count="12">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A32:J32"/>
     <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A32:J32"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:J3"/>
@@ -6548,50 +6515,42 @@
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1">
-      <c r="A8" s="24" t="n">
+      <c r="A8" s="66" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>Inj. Xone</t>
         </is>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="68" t="inlineStr">
         <is>
           <t>Ceftriaxone</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I8" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J8" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D8" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E8" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="69" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="G8" s="69" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="H8" s="69" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="I8" s="69" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="J8" s="68" t="inlineStr">
+        <is>
+          <t>SL16 / SSB S000068</t>
         </is>
       </c>
     </row>
@@ -6836,50 +6795,42 @@
       </c>
     </row>
     <row r="15" ht="13.5" customHeight="1">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="66" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="40" t="inlineStr">
+      <c r="B15" s="68" t="inlineStr">
         <is>
           <t>Inj. Tramadol</t>
         </is>
       </c>
-      <c r="C15" s="40" t="inlineStr">
+      <c r="C15" s="68" t="inlineStr">
         <is>
           <t>Tramadol</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J15" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D15" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E15" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="69" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="G15" s="69" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="H15" s="69" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="I15" s="69" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="J15" s="68" t="inlineStr">
+        <is>
+          <t>SL25 / SSB S000135</t>
         </is>
       </c>
     </row>
@@ -7155,11 +7106,11 @@
       <c r="E23" s="62" t="n"/>
       <c r="F23" s="62" t="n"/>
       <c r="G23" s="63" t="n">
-        <v>1447.58</v>
+        <v>1526.78</v>
       </c>
       <c r="H23" s="43" t="n"/>
-      <c r="I23" s="42" t="n">
-        <v>975.1799999999999</v>
+      <c r="I23" s="63" t="n">
+        <v>1005.65</v>
       </c>
       <c r="J23" s="43" t="n"/>
     </row>
@@ -7280,11 +7231,11 @@
       <c r="E31" s="59" t="n"/>
       <c r="F31" s="59" t="n"/>
       <c r="G31" s="64" t="n">
-        <v>3947.58</v>
+        <v>4026.78</v>
       </c>
       <c r="H31" s="65" t="inlineStr">
         <is>
-          <t>Total Cost: ₹975.18  |  Margin: ₹2,972.40</t>
+          <t>Total Cost: ₹1,005.65  |  Margin: ₹3,021.13</t>
         </is>
       </c>
       <c r="I31" s="59" t="n"/>
@@ -7299,15 +7250,14 @@
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 2 item(s) without MRP: Inj. Tramadol | Inj. Xone</t>
+      <c r="A34" s="70" t="inlineStr">
+        <is>
+          <t>✓ All items now priced from Master Rate Card — no missing MRPs</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A25:J25"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="I2:J2"/>
@@ -7315,10 +7265,11 @@
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A33:J33"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="A28:J28"/>
-    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A25:J25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -8128,50 +8079,42 @@
       </c>
     </row>
     <row r="22" ht="13.5" customHeight="1">
-      <c r="A22" s="24" t="n">
+      <c r="A22" s="66" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="40" t="inlineStr">
+      <c r="B22" s="68" t="inlineStr">
         <is>
           <t>Plain Sheet</t>
         </is>
       </c>
-      <c r="C22" s="40" t="inlineStr">
+      <c r="C22" s="68" t="inlineStr">
         <is>
           <t>Draping sheet</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="n">
+      <c r="D22" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E22" s="66" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G22" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H22" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I22" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J22" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="F22" s="69" t="n">
+        <v>200</v>
+      </c>
+      <c r="G22" s="69" t="n">
+        <v>400</v>
+      </c>
+      <c r="H22" s="69" t="n">
+        <v>65</v>
+      </c>
+      <c r="I22" s="69" t="n">
+        <v>130</v>
+      </c>
+      <c r="J22" s="68" t="inlineStr">
+        <is>
+          <t>SL83 / BP Pharma #248/#288</t>
         </is>
       </c>
     </row>
@@ -8464,50 +8407,42 @@
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1">
-      <c r="A30" s="24" t="n">
+      <c r="A30" s="66" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="40" t="inlineStr">
+      <c r="B30" s="68" t="inlineStr">
         <is>
           <t>Vacuum Suck</t>
         </is>
       </c>
-      <c r="C30" s="40" t="inlineStr">
+      <c r="C30" s="68" t="inlineStr">
         <is>
           <t>Vacuum suction</t>
         </is>
       </c>
-      <c r="D30" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E30" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G30" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H30" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I30" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J30" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D30" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E30" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="69" t="n">
+        <v>543</v>
+      </c>
+      <c r="G30" s="69" t="n">
+        <v>543</v>
+      </c>
+      <c r="H30" s="69" t="n">
+        <v>50</v>
+      </c>
+      <c r="I30" s="69" t="n">
+        <v>50</v>
+      </c>
+      <c r="J30" s="68" t="inlineStr">
+        <is>
+          <t>SL102 Suction Tube VACCU / Perfia</t>
         </is>
       </c>
     </row>
@@ -8724,98 +8659,90 @@
       </c>
     </row>
     <row r="36" ht="13.5" customHeight="1">
-      <c r="A36" s="24" t="n">
+      <c r="A36" s="66" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="40" t="inlineStr">
+      <c r="B36" s="68" t="inlineStr">
         <is>
           <t>Blade No. 10</t>
         </is>
       </c>
-      <c r="C36" s="40" t="inlineStr">
+      <c r="C36" s="68" t="inlineStr">
         <is>
           <t>Surgical blade</t>
         </is>
       </c>
-      <c r="D36" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E36" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="41" t="inlineStr">
+      <c r="D36" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E36" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="69" t="n">
+        <v>750</v>
+      </c>
+      <c r="G36" s="69" t="n">
+        <v>750</v>
+      </c>
+      <c r="H36" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="G36" s="41" t="inlineStr">
+      <c r="I36" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="H36" s="41" t="inlineStr">
+      <c r="J36" s="68" t="inlineStr">
+        <is>
+          <t>SL81 / Stock file</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="13.5" customHeight="1">
+      <c r="A37" s="66" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="68" t="inlineStr">
+        <is>
+          <t>Blade No. 20</t>
+        </is>
+      </c>
+      <c r="C37" s="68" t="inlineStr">
+        <is>
+          <t>Surgical blade</t>
+        </is>
+      </c>
+      <c r="D37" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E37" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="69" t="n">
+        <v>710</v>
+      </c>
+      <c r="G37" s="69" t="n">
+        <v>710</v>
+      </c>
+      <c r="H37" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="I36" s="41" t="inlineStr">
+      <c r="I37" s="69" t="inlineStr">
         <is>
           <t>⚠</t>
         </is>
       </c>
-      <c r="J36" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="13.5" customHeight="1">
-      <c r="A37" s="24" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="40" t="inlineStr">
-        <is>
-          <t>Blade No. 20</t>
-        </is>
-      </c>
-      <c r="C37" s="40" t="inlineStr">
-        <is>
-          <t>Surgical blade</t>
-        </is>
-      </c>
-      <c r="D37" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E37" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G37" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H37" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I37" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J37" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="J37" s="68" t="inlineStr">
+        <is>
+          <t>SL82 / Stock file</t>
         </is>
       </c>
     </row>
@@ -9531,11 +9458,11 @@
       <c r="E56" s="62" t="n"/>
       <c r="F56" s="62" t="n"/>
       <c r="G56" s="63" t="n">
-        <v>8107.76</v>
+        <v>10510.76</v>
       </c>
       <c r="H56" s="43" t="n"/>
-      <c r="I56" s="42" t="n">
-        <v>4595.19</v>
+      <c r="I56" s="63" t="n">
+        <v>4775.19</v>
       </c>
       <c r="J56" s="43" t="n"/>
     </row>
@@ -9656,11 +9583,11 @@
       <c r="E64" s="59" t="n"/>
       <c r="F64" s="59" t="n"/>
       <c r="G64" s="64" t="n">
-        <v>10607.76</v>
+        <v>13010.76</v>
       </c>
       <c r="H64" s="65" t="inlineStr">
         <is>
-          <t>Total Cost: ₹4,595.19  |  Margin: ₹6,012.57</t>
+          <t>Total Cost: ₹4,775.19  |  Margin: ₹8,235.57</t>
         </is>
       </c>
       <c r="I64" s="59" t="n"/>
@@ -9675,9 +9602,9 @@
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 8 item(s) without MRP: Sanitary Pad | Cord Clamp | Blade No. 10 | W9932 | Inj. Campuse 2acs | Plain Sheet | Blade No. 20 | Vacuum Suck</t>
+      <c r="A67" s="70" t="inlineStr">
+        <is>
+          <t>⚠ 4 item(s) without MRP: Inj. Campuse 2acs | Sanitary Pad | W9932 | Cord Clamp</t>
         </is>
       </c>
     </row>
@@ -10008,46 +9935,38 @@
       </c>
     </row>
     <row r="10" ht="13.5" customHeight="1">
-      <c r="A10" s="24" t="n">
+      <c r="A10" s="66" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B10" s="68" t="inlineStr">
         <is>
           <t>2ml Syringe</t>
         </is>
       </c>
-      <c r="C10" s="40" t="n"/>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="n">
+      <c r="C10" s="68" t="n"/>
+      <c r="D10" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E10" s="66" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G10" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H10" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I10" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J10" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="F10" s="69" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="G10" s="69" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="H10" s="69" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="I10" s="69" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="J10" s="68" t="inlineStr">
+        <is>
+          <t>SL58 / SSB S000069</t>
         </is>
       </c>
     </row>
@@ -10208,94 +10127,78 @@
       </c>
     </row>
     <row r="15" ht="13.5" customHeight="1">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="66" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="40" t="inlineStr">
+      <c r="B15" s="68" t="inlineStr">
         <is>
           <t>Inj. Tramadol 50mg</t>
         </is>
       </c>
-      <c r="C15" s="40" t="inlineStr">
+      <c r="C15" s="68" t="inlineStr">
         <is>
           <t>Analgesic</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J15" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D15" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E15" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="69" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="G15" s="69" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="H15" s="69" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="I15" s="69" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="J15" s="68" t="inlineStr">
+        <is>
+          <t>SL25 / SSB S000135</t>
         </is>
       </c>
     </row>
     <row r="16" ht="13.5" customHeight="1">
-      <c r="A16" s="24" t="n">
+      <c r="A16" s="66" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B16" s="68" t="inlineStr">
         <is>
           <t>100ml NS</t>
         </is>
       </c>
-      <c r="C16" s="40" t="n"/>
-      <c r="D16" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G16" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H16" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I16" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J16" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="C16" s="68" t="n"/>
+      <c r="D16" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E16" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="G16" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="H16" s="69" t="n">
+        <v>13</v>
+      </c>
+      <c r="I16" s="69" t="n">
+        <v>13</v>
+      </c>
+      <c r="J16" s="68" t="inlineStr">
+        <is>
+          <t>SL3 / Vivek F-748</t>
         </is>
       </c>
     </row>
@@ -10715,11 +10618,11 @@
       <c r="E27" s="62" t="n"/>
       <c r="F27" s="62" t="n"/>
       <c r="G27" s="63" t="n">
-        <v>2275.46</v>
+        <v>2321.1</v>
       </c>
       <c r="H27" s="43" t="n"/>
-      <c r="I27" s="42" t="n">
-        <v>971.1799999999999</v>
+      <c r="I27" s="63" t="n">
+        <v>992.74</v>
       </c>
       <c r="J27" s="43" t="n"/>
     </row>
@@ -10840,11 +10743,11 @@
       <c r="E35" s="59" t="n"/>
       <c r="F35" s="59" t="n"/>
       <c r="G35" s="64" t="n">
-        <v>4775.46</v>
+        <v>4821.1</v>
       </c>
       <c r="H35" s="65" t="inlineStr">
         <is>
-          <t>Total Cost: ₹971.18  |  Margin: ₹3,804.28</t>
+          <t>Total Cost: ₹992.74  |  Margin: ₹3,828.36</t>
         </is>
       </c>
       <c r="I35" s="59" t="n"/>
@@ -10859,9 +10762,9 @@
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 5 item(s) without MRP: 2ml Syringe | Inj. Tramadol 50mg | Cap + Mask | T.U.R.P. Set | 100ml NS</t>
+      <c r="A38" s="70" t="inlineStr">
+        <is>
+          <t>⚠ 2 item(s) without MRP: T.U.R.P. Set | Cap + Mask</t>
         </is>
       </c>
     </row>
@@ -10869,8 +10772,8 @@
   <mergeCells count="12">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A32:J32"/>
     <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A32:J32"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:J3"/>
@@ -13948,50 +13851,42 @@
       </c>
     </row>
     <row r="15" ht="13.5" customHeight="1">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="66" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="40" t="inlineStr">
+      <c r="B15" s="68" t="inlineStr">
         <is>
           <t>Inj. Sensoricaine (Heavy)</t>
         </is>
       </c>
-      <c r="C15" s="40" t="inlineStr">
+      <c r="C15" s="68" t="inlineStr">
         <is>
           <t>Bupivacaine Heavy</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="I15" s="41" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="J15" s="40" t="inlineStr">
-        <is>
-          <t>⚠ MRP NOT FOUND — fill in manually</t>
+      <c r="D15" s="66" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="E15" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="69" t="n">
+        <v>31.47</v>
+      </c>
+      <c r="G15" s="69" t="n">
+        <v>31.47</v>
+      </c>
+      <c r="H15" s="69" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="I15" s="69" t="n">
+        <v>24.76</v>
+      </c>
+      <c r="J15" s="68" t="inlineStr">
+        <is>
+          <t>SL7 Anawin Heavy / SSB S000092</t>
         </is>
       </c>
     </row>
@@ -14358,12 +14253,12 @@
       <c r="D25" s="62" t="n"/>
       <c r="E25" s="62" t="n"/>
       <c r="F25" s="62" t="n"/>
-      <c r="G25" s="42" t="n">
-        <v>2388.86</v>
+      <c r="G25" s="63" t="n">
+        <v>2420.33</v>
       </c>
       <c r="H25" s="43" t="n"/>
-      <c r="I25" s="42" t="n">
-        <v>785.95</v>
+      <c r="I25" s="63" t="n">
+        <v>810.71</v>
       </c>
       <c r="J25" s="43" t="n"/>
     </row>
@@ -14483,12 +14378,12 @@
       <c r="D33" s="59" t="n"/>
       <c r="E33" s="59" t="n"/>
       <c r="F33" s="59" t="n"/>
-      <c r="G33" s="52" t="n">
-        <v>4888.86</v>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>Total Cost: ₹785.95  |  Margin: ₹4,102.91</t>
+      <c r="G33" s="64" t="n">
+        <v>4920.33</v>
+      </c>
+      <c r="H33" s="65" t="inlineStr">
+        <is>
+          <t>Total Cost: ₹810.71  |  Margin: ₹4,109.62</t>
         </is>
       </c>
       <c r="I33" s="59" t="n"/>
@@ -14503,9 +14398,9 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 1 item(s) without MRP: Inj. Sensoricaine (Heavy)</t>
+      <c r="A36" s="70" t="inlineStr">
+        <is>
+          <t>✓ All items now priced from Master Rate Card — no missing MRPs</t>
         </is>
       </c>
     </row>
@@ -16275,15 +16170,14 @@
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>⚠ 3 item(s) without MRP: Pulse Oximeter | O2 | Cardiac Monitor</t>
+      <c r="A34" s="70" t="inlineStr">
+        <is>
+          <t>⚠ 3 item(s) without MRP: O2 | Cardiac Monitor | Pulse Oximeter</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A25:J25"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="I2:J2"/>
@@ -16291,10 +16185,11 @@
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A34:J34"/>
+    <mergeCell ref="A33:J33"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="A28:J28"/>
-    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A25:J25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>